<commit_message>
docs: update Gantt chart progress and rewrite prototype report
- Gantt chart: mark completed backend/verification/marketplace/CI tasks
  done, move Today marker to 9/14/2026, adjust dates to reflect actual
  completion timeline
- prototype report: rewritten as a report-class LaTeX document (chapters,
  table of contents, TikZ architecture/pipeline diagrams, metrics table,
  bibliography) matching the course reference template, with real content
  pulled from the current schema, rule engine, and test results

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Deadstock_Gantt_Chart.xlsx
+++ b/docs/Deadstock_Gantt_Chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Puria\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Puria\Deadstock-Management-Stock\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{617D4E93-8928-4FE8-A98D-304F308DC34C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90CD607F-BF76-469B-AFA5-9299B3F16193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProjectSchedule" sheetId="11" r:id="rId1"/>
@@ -215,9 +215,6 @@
     <t>Data Store Schema Design (Vendors, Buyers, Inventory, Verification, Listings, Transactions)</t>
   </si>
   <si>
-    <t>CI Pipeline Setup (build, unit tests, lint)</t>
-  </si>
-  <si>
     <t>API / Endpoint Planning (Vendor to Buyer workflow)</t>
   </si>
   <si>
@@ -261,6 +258,9 @@
   </si>
   <si>
     <t>Project Submission &amp; Demo</t>
+  </si>
+  <si>
+    <t>CI Pipeline Setup &amp; Prototype Stage Report/Deck</t>
   </si>
 </sst>
 </file>
@@ -1587,21 +1587,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BL45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" customWidth="1"/>
-    <col min="7" max="7" width="2.7109375" customWidth="1"/>
-    <col min="8" max="8" width="6.140625" hidden="1" customWidth="1"/>
-    <col min="9" max="64" width="2.5703125" customWidth="1"/>
-    <col min="69" max="70" width="10.28515625"/>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.88671875" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" customWidth="1"/>
+    <col min="5" max="5" width="10.44140625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" customWidth="1"/>
+    <col min="7" max="7" width="2.6640625" customWidth="1"/>
+    <col min="8" max="8" width="6.109375" hidden="1" customWidth="1"/>
+    <col min="9" max="64" width="2.5546875" customWidth="1"/>
+    <col min="69" max="70" width="10.33203125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:64" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:64" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="B1" s="16" t="s">
         <v>24</v>
       </c>
@@ -1633,7 +1633,7 @@
       <c r="Z1" s="106"/>
       <c r="AA1" s="106"/>
     </row>
-    <row r="2" spans="1:64" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:64" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="9" t="s">
         <v>25</v>
       </c>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="F2" s="102"/>
     </row>
-    <row r="3" spans="1:64" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:64" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="9" t="s">
         <v>26</v>
       </c>
@@ -1653,11 +1653,11 @@
         <v>22</v>
       </c>
       <c r="E3" s="101">
-        <v>46272</v>
+        <v>46279</v>
       </c>
       <c r="F3" s="102"/>
     </row>
-    <row r="4" spans="1:64" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:64" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D4" s="6" t="s">
         <v>8</v>
       </c>
@@ -1745,7 +1745,7 @@
       <c r="BK4" s="104"/>
       <c r="BL4" s="105"/>
     </row>
-    <row r="5" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="G5" s="6"/>
       <c r="I5" s="13">
@@ -1973,7 +1973,7 @@
         <v>46292</v>
       </c>
     </row>
-    <row r="6" spans="1:64" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:64" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19"/>
       <c r="B6" s="10" t="s">
         <v>9</v>
@@ -2219,7 +2219,7 @@
         <v>S</v>
       </c>
     </row>
-    <row r="7" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19"/>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -2288,7 +2288,7 @@
       <c r="BK7" s="82"/>
       <c r="BL7" s="82"/>
     </row>
-    <row r="8" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19"/>
       <c r="B8" s="26" t="s">
         <v>27</v>
@@ -2359,7 +2359,7 @@
       <c r="BK8" s="82"/>
       <c r="BL8" s="82"/>
     </row>
-    <row r="9" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19"/>
       <c r="B9" s="31" t="s">
         <v>28</v>
@@ -2438,7 +2438,7 @@
       <c r="BK9" s="82"/>
       <c r="BL9" s="82"/>
     </row>
-    <row r="10" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19"/>
       <c r="B10" s="31" t="s">
         <v>30</v>
@@ -2517,7 +2517,7 @@
       <c r="BK10" s="82"/>
       <c r="BL10" s="82"/>
     </row>
-    <row r="11" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="19"/>
       <c r="B11" s="31" t="s">
         <v>32</v>
@@ -2596,7 +2596,7 @@
       <c r="BK11" s="82"/>
       <c r="BL11" s="82"/>
     </row>
-    <row r="12" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19"/>
       <c r="B12" s="31" t="s">
         <v>33</v>
@@ -2675,7 +2675,7 @@
       <c r="BK12" s="82"/>
       <c r="BL12" s="82"/>
     </row>
-    <row r="13" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="19"/>
       <c r="B13" s="31" t="s">
         <v>34</v>
@@ -2754,7 +2754,7 @@
       <c r="BK13" s="82"/>
       <c r="BL13" s="82"/>
     </row>
-    <row r="14" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="19"/>
       <c r="B14" s="36" t="s">
         <v>35</v>
@@ -2825,7 +2825,7 @@
       <c r="BK14" s="82"/>
       <c r="BL14" s="82"/>
     </row>
-    <row r="15" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19"/>
       <c r="B15" s="41" t="s">
         <v>36</v>
@@ -2904,7 +2904,7 @@
       <c r="BK15" s="82"/>
       <c r="BL15" s="82"/>
     </row>
-    <row r="16" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="19"/>
       <c r="B16" s="41" t="s">
         <v>37</v>
@@ -2983,7 +2983,7 @@
       <c r="BK16" s="82"/>
       <c r="BL16" s="82"/>
     </row>
-    <row r="17" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19"/>
       <c r="B17" s="41" t="s">
         <v>39</v>
@@ -2992,7 +2992,7 @@
         <v>38</v>
       </c>
       <c r="D17" s="43">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E17" s="44">
         <v>46258</v>
@@ -3062,7 +3062,7 @@
       <c r="BK17" s="82"/>
       <c r="BL17" s="82"/>
     </row>
-    <row r="18" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="19"/>
       <c r="B18" s="41" t="s">
         <v>40</v>
@@ -3141,7 +3141,7 @@
       <c r="BK18" s="82"/>
       <c r="BL18" s="82"/>
     </row>
-    <row r="19" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="19"/>
       <c r="B19" s="41" t="s">
         <v>42</v>
@@ -3220,7 +3220,7 @@
       <c r="BK19" s="82"/>
       <c r="BL19" s="82"/>
     </row>
-    <row r="20" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="19"/>
       <c r="B20" s="46" t="s">
         <v>43</v>
@@ -3291,7 +3291,7 @@
       <c r="BK20" s="82"/>
       <c r="BL20" s="82"/>
     </row>
-    <row r="21" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="19"/>
       <c r="B21" s="51" t="s">
         <v>44</v>
@@ -3300,18 +3300,18 @@
         <v>31</v>
       </c>
       <c r="D21" s="53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" s="54">
-        <v>46279</v>
+        <v>46272</v>
       </c>
       <c r="F21" s="55">
-        <v>46285</v>
+        <v>46273</v>
       </c>
       <c r="G21" s="25"/>
       <c r="H21" s="25">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I21" s="82"/>
       <c r="J21" s="82"/>
@@ -3370,27 +3370,27 @@
       <c r="BK21" s="82"/>
       <c r="BL21" s="82"/>
     </row>
-    <row r="22" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="19"/>
       <c r="B22" s="51" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="C22" s="52" t="s">
         <v>41</v>
       </c>
       <c r="D22" s="53">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E22" s="54">
         <v>46272</v>
       </c>
       <c r="F22" s="55">
-        <v>46285</v>
+        <v>46278</v>
       </c>
       <c r="G22" s="25"/>
       <c r="H22" s="25">
         <f t="shared" si="6"/>
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I22" s="82"/>
       <c r="J22" s="82"/>
@@ -3449,27 +3449,27 @@
       <c r="BK22" s="82"/>
       <c r="BL22" s="82"/>
     </row>
-    <row r="23" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19"/>
       <c r="B23" s="51" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C23" s="52" t="s">
         <v>31</v>
       </c>
       <c r="D23" s="53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" s="54">
-        <v>46286</v>
+        <v>46273</v>
       </c>
       <c r="F23" s="55">
-        <v>46292</v>
+        <v>46275</v>
       </c>
       <c r="G23" s="25"/>
       <c r="H23" s="25">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I23" s="82"/>
       <c r="J23" s="82"/>
@@ -3528,27 +3528,27 @@
       <c r="BK23" s="82"/>
       <c r="BL23" s="82"/>
     </row>
-    <row r="24" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="19"/>
       <c r="B24" s="51" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C24" s="52" t="s">
         <v>38</v>
       </c>
       <c r="D24" s="53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="54">
-        <v>46286</v>
+        <v>46274</v>
       </c>
       <c r="F24" s="55">
-        <v>46292</v>
+        <v>46275</v>
       </c>
       <c r="G24" s="25"/>
       <c r="H24" s="25">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I24" s="82"/>
       <c r="J24" s="82"/>
@@ -3607,19 +3607,19 @@
       <c r="BK24" s="82"/>
       <c r="BL24" s="82"/>
     </row>
-    <row r="25" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="19"/>
       <c r="B25" s="51" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C25" s="52" t="s">
         <v>29</v>
       </c>
       <c r="D25" s="53">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="E25" s="54">
-        <v>46293</v>
+        <v>46276</v>
       </c>
       <c r="F25" s="55">
         <v>46299</v>
@@ -3627,7 +3627,7 @@
       <c r="G25" s="25"/>
       <c r="H25" s="25">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="I25" s="82"/>
       <c r="J25" s="82"/>
@@ -3686,10 +3686,10 @@
       <c r="BK25" s="82"/>
       <c r="BL25" s="82"/>
     </row>
-    <row r="26" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="19"/>
       <c r="B26" s="56" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C26" s="57"/>
       <c r="D26" s="58"/>
@@ -3757,27 +3757,27 @@
       <c r="BK26" s="82"/>
       <c r="BL26" s="82"/>
     </row>
-    <row r="27" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="19"/>
       <c r="B27" s="61" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C27" s="62" t="s">
         <v>31</v>
       </c>
       <c r="D27" s="63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" s="64">
-        <v>46300</v>
+        <v>46274</v>
       </c>
       <c r="F27" s="65">
-        <v>46306</v>
+        <v>46278</v>
       </c>
       <c r="G27" s="25"/>
       <c r="H27" s="25">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I27" s="82"/>
       <c r="J27" s="82"/>
@@ -3836,27 +3836,27 @@
       <c r="BK27" s="82"/>
       <c r="BL27" s="82"/>
     </row>
-    <row r="28" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="19"/>
       <c r="B28" s="61" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C28" s="62" t="s">
         <v>38</v>
       </c>
       <c r="D28" s="63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" s="64">
-        <v>46307</v>
+        <v>46275</v>
       </c>
       <c r="F28" s="65">
-        <v>46313</v>
+        <v>46278</v>
       </c>
       <c r="G28" s="25"/>
       <c r="H28" s="25">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I28" s="82"/>
       <c r="J28" s="82"/>
@@ -3915,27 +3915,27 @@
       <c r="BK28" s="82"/>
       <c r="BL28" s="82"/>
     </row>
-    <row r="29" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="19"/>
       <c r="B29" s="61" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C29" s="62" t="s">
         <v>41</v>
       </c>
       <c r="D29" s="63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" s="64">
-        <v>46314</v>
+        <v>46275</v>
       </c>
       <c r="F29" s="65">
-        <v>46320</v>
+        <v>46278</v>
       </c>
       <c r="G29" s="25"/>
       <c r="H29" s="25">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I29" s="82"/>
       <c r="J29" s="82"/>
@@ -3994,10 +3994,10 @@
       <c r="BK29" s="82"/>
       <c r="BL29" s="82"/>
     </row>
-    <row r="30" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="19"/>
       <c r="B30" s="61" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C30" s="62" t="s">
         <v>29</v>
@@ -4073,19 +4073,19 @@
       <c r="BK30" s="82"/>
       <c r="BL30" s="82"/>
     </row>
-    <row r="31" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="19"/>
       <c r="B31" s="61" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C31" s="62" t="s">
         <v>41</v>
       </c>
       <c r="D31" s="63">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E31" s="64">
-        <v>46328</v>
+        <v>46276</v>
       </c>
       <c r="F31" s="65">
         <v>46334</v>
@@ -4093,7 +4093,7 @@
       <c r="G31" s="25"/>
       <c r="H31" s="25">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>59</v>
       </c>
       <c r="I31" s="82"/>
       <c r="J31" s="82"/>
@@ -4152,10 +4152,10 @@
       <c r="BK31" s="82"/>
       <c r="BL31" s="82"/>
     </row>
-    <row r="32" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="19"/>
       <c r="B32" s="66" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C32" s="67"/>
       <c r="D32" s="68"/>
@@ -4223,27 +4223,27 @@
       <c r="BK32" s="82"/>
       <c r="BL32" s="82"/>
     </row>
-    <row r="33" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="19"/>
       <c r="B33" s="71" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C33" s="72" t="s">
         <v>38</v>
       </c>
       <c r="D33" s="73">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" s="74">
-        <v>46335</v>
+        <v>46275</v>
       </c>
       <c r="F33" s="75">
-        <v>46341</v>
+        <v>46278</v>
       </c>
       <c r="G33" s="25"/>
       <c r="H33" s="25">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I33" s="82"/>
       <c r="J33" s="82"/>
@@ -4302,19 +4302,19 @@
       <c r="BK33" s="82"/>
       <c r="BL33" s="82"/>
     </row>
-    <row r="34" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="19"/>
       <c r="B34" s="71" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C34" s="72" t="s">
         <v>29</v>
       </c>
       <c r="D34" s="73">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E34" s="74">
-        <v>46342</v>
+        <v>46276</v>
       </c>
       <c r="F34" s="75">
         <v>46348</v>
@@ -4322,7 +4322,7 @@
       <c r="G34" s="25"/>
       <c r="H34" s="25">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>73</v>
       </c>
       <c r="I34" s="82"/>
       <c r="J34" s="82"/>
@@ -4381,10 +4381,10 @@
       <c r="BK34" s="82"/>
       <c r="BL34" s="82"/>
     </row>
-    <row r="35" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="19"/>
       <c r="B35" s="71" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C35" s="72" t="s">
         <v>31</v>
@@ -4460,10 +4460,10 @@
       <c r="BK35" s="82"/>
       <c r="BL35" s="82"/>
     </row>
-    <row r="36" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="19"/>
       <c r="B36" s="71" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C36" s="72" t="s">
         <v>29</v>
@@ -4539,10 +4539,10 @@
       <c r="BK36" s="82"/>
       <c r="BL36" s="82"/>
     </row>
-    <row r="37" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="19"/>
       <c r="B37" s="71" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C37" s="72" t="s">
         <v>29</v>
@@ -4618,7 +4618,7 @@
       <c r="BK37" s="82"/>
       <c r="BL37" s="82"/>
     </row>
-    <row r="38" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="19"/>
       <c r="B38" s="20"/>
       <c r="C38" s="21"/>
@@ -4687,7 +4687,7 @@
       <c r="BK38" s="82"/>
       <c r="BL38" s="82"/>
     </row>
-    <row r="39" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="19"/>
       <c r="B39" s="20"/>
       <c r="C39" s="21"/>
@@ -4756,7 +4756,7 @@
       <c r="BK39" s="82"/>
       <c r="BL39" s="82"/>
     </row>
-    <row r="40" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="19"/>
       <c r="B40" s="20"/>
       <c r="C40" s="21"/>
@@ -4825,7 +4825,7 @@
       <c r="BK40" s="82"/>
       <c r="BL40" s="82"/>
     </row>
-    <row r="41" spans="1:64" s="3" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:64" s="3" customFormat="1" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="19"/>
       <c r="B41" s="76" t="s">
         <v>0</v>
@@ -4896,11 +4896,11 @@
       <c r="BK41" s="84"/>
       <c r="BL41" s="84"/>
     </row>
-    <row r="42" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:64" x14ac:dyDescent="0.3">
       <c r="A42" s="6"/>
       <c r="G42" s="6"/>
     </row>
-    <row r="43" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:64" x14ac:dyDescent="0.3">
       <c r="B43" s="17" t="s">
         <v>12</v>
       </c>
@@ -4909,13 +4909,13 @@
         <v>43113</v>
       </c>
     </row>
-    <row r="44" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:64" x14ac:dyDescent="0.3">
       <c r="B44" s="99" t="s">
         <v>17</v>
       </c>
       <c r="C44" s="18"/>
     </row>
-    <row r="45" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:64" x14ac:dyDescent="0.3">
       <c r="B45" s="98" t="s">
         <v>23</v>
       </c>
@@ -5001,103 +5001,103 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:C22"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.85546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="87.140625" style="85" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="2.88671875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="87.109375" style="85" customWidth="1"/>
+    <col min="3" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="2:3" s="87" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:3" s="87" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="86" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="86"/>
     </row>
-    <row r="3" spans="2:3" s="89" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:3" s="89" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="88" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="88"/>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="97" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="2:3" s="90" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:3" s="90" customFormat="1" ht="25.8" x14ac:dyDescent="0.5">
       <c r="B6" s="92" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="60" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B7" s="93" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B8" s="91"/>
     </row>
-    <row r="9" spans="2:3" s="90" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:3" s="90" customFormat="1" ht="25.8" x14ac:dyDescent="0.5">
       <c r="B9" s="92" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="60" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B10" s="93" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B11" s="94" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B12" s="91"/>
     </row>
-    <row r="13" spans="2:3" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B13" s="100" t="str">
         <f>HYPERLINK("https://vertex42.link/HowToMakeAGanttChart","► Watch How This Gantt Chart Was Created")</f>
         <v>► Watch How This Gantt Chart Was Created</v>
       </c>
     </row>
-    <row r="14" spans="2:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B14" s="91"/>
     </row>
-    <row r="15" spans="2:3" s="90" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:3" s="90" customFormat="1" ht="25.8" x14ac:dyDescent="0.5">
       <c r="B15" s="92" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="2:3" ht="30" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B16" s="93" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="2:2" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B17" s="94" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="2:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B18" s="91"/>
     </row>
-    <row r="19" spans="2:2" s="90" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:2" s="90" customFormat="1" ht="25.8" x14ac:dyDescent="0.5">
       <c r="B19" s="92" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="2:2" ht="60" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B20" s="93" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="2:2" ht="15" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B21" s="91"/>
     </row>
-    <row r="22" spans="2:2" ht="75" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:2" ht="72" x14ac:dyDescent="0.3">
       <c r="B22" s="93" t="s">
         <v>16</v>
       </c>

</xml_diff>